<commit_message>
Updated the pdf to text extractor
</commit_message>
<xml_diff>
--- a/output/invoices.xlsx
+++ b/output/invoices.xlsx
@@ -413,36 +413,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>invoice_no</t>
+          <t>Invoice Date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>invoice_date</t>
+          <t>Invoice Number</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>gstin</t>
+          <t>Invoice Total</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>buyer_pan</t>
+          <t>Billing Address</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>total</t>
+          <t>Due Date</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Referene No.</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>CST value</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Delivery_and_Billing_Period</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Item Total</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>File Path</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>source_file</t>
         </is>
@@ -451,30 +501,80 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>30.11.2025</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>3251202779</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>30.11.2025</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>37AAACR5055K2Z5</t>
+          <t>1,409,394.03</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AAACI1681G</t>
+          <t>VIDYUT NAGAR ,GAUTUM BHUDDHA ,DADRI ,  201008 ,Uttar Pradesh</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1,409,394.03</t>
+          <t>05.12.2025</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>INDIAN OIL CORPORATION LIMITED  DADRI</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CTR-690</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.720</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>27,635.18</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>16.11.2025 to 30.11.2025</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1,381,758.85</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1,42,156.26</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>invoices\sample1.pdf</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>sample1.pdf</t>
         </is>
@@ -483,32 +583,246 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>30.11.2025</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>3251202766</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3,509,607.11</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PANIPAT VILLAGE, ,BOHALI ,PANIPAT ,  132103 ,Haryana</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>INDIAN OIL CORPORATION LIMITED  PANIPAT REFINERY,</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CTR-635</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>9.720</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>68,815.83</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>16.11.2025 to 30.11.2025</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>3,440,791.28</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>3,53,990.87</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>invoices\sample2.pdf</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>sample2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>30.11.2025</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>AAACI1681G</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>3,509,607.11</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>sample2.pdf</t>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3255202766</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1,754,540.34</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PANIPAT VILLAGE, ,BOHALI ,PANIPAT ,  132103 ,Haryana</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>INDIAN OIL CORPORATION LIMITED  PANIPAT REFINERY,</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CTR-635</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>9.720</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>34,402.75</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>16.11.2025 to 30.11.2025</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1,720,137.59</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1,76,968.89</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>invoices\sample3.pdf</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>sample3.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30.11.2025</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3255202779</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>704,591.32</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>VIDYUT NAGAR ,GAUTUM BHUDDHA ,DADRI ,  201008 ,Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>INDIAN OIL CORPORATION LIMITED  DADRI</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CTR-690</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>9.720</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>13,815.52</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>16.11.2025 to 30.11.2025</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>690,775.80</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>71,067.47</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>invoices\sample4.pdf</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>sample4.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Generalize invoice parsing extraction logic and clean up temporary files
</commit_message>
<xml_diff>
--- a/output/invoices.xlsx
+++ b/output/invoices.xlsx
@@ -7007,7 +7007,11 @@
           <t>CTR-1246</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>1246</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -7110,7 +7114,11 @@
           <t>CTR-1246</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>1246</t>
+        </is>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -7213,7 +7221,11 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>635</t>
+        </is>
+      </c>
       <c r="J64" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -7316,7 +7328,11 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>635</t>
+        </is>
+      </c>
       <c r="J65" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -7419,7 +7435,11 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>690</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -7430,7 +7450,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M66" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7518,7 +7542,11 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>690</t>
+        </is>
+      </c>
       <c r="J67" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -7529,7 +7557,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7617,7 +7649,11 @@
           <t>CTR-691</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
       <c r="J68" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -7628,7 +7664,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M68" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7716,7 +7756,11 @@
           <t>CTR-691</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>691</t>
+        </is>
+      </c>
       <c r="J69" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -7727,7 +7771,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7815,7 +7863,11 @@
           <t>CTR-692</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
       <c r="J70" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -7826,7 +7878,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7914,7 +7970,11 @@
           <t>CTR-692</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
       <c r="J71" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -7925,7 +7985,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8013,7 +8077,11 @@
           <t>CTR-693</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>693</t>
+        </is>
+      </c>
       <c r="J72" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -8116,7 +8184,11 @@
           <t>CTR-693</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>693</t>
+        </is>
+      </c>
       <c r="J73" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -8219,7 +8291,11 @@
           <t>CTR-694</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>694</t>
+        </is>
+      </c>
       <c r="J74" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -8322,7 +8398,11 @@
           <t>CTR-694</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>694</t>
+        </is>
+      </c>
       <c r="J75" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -8425,7 +8505,11 @@
           <t>CTR-716</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>716</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -8436,7 +8520,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr"/>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M76" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8524,7 +8612,11 @@
           <t>CTR-716</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>716</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -8535,7 +8627,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M77" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8623,7 +8719,11 @@
           <t>CTR-717</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>717</t>
+        </is>
+      </c>
       <c r="J78" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -8634,7 +8734,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M78" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8722,7 +8826,11 @@
           <t>CTR-717</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>717</t>
+        </is>
+      </c>
       <c r="J79" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -8733,7 +8841,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M79" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8821,7 +8933,11 @@
           <t>CTR-718</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>718</t>
+        </is>
+      </c>
       <c r="J80" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -8832,7 +8948,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M80" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8920,7 +9040,11 @@
           <t>CTR-718</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>718</t>
+        </is>
+      </c>
       <c r="J81" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -8931,7 +9055,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M81" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9019,7 +9147,11 @@
           <t>CTR-719</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>719</t>
+        </is>
+      </c>
       <c r="J82" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -9030,7 +9162,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M82" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9118,7 +9254,11 @@
           <t>CTR-719</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>719</t>
+        </is>
+      </c>
       <c r="J83" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -9129,7 +9269,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M83" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9217,7 +9361,11 @@
           <t>CTR-720</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
       <c r="J84" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -9228,7 +9376,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>23AAACI1681G1ZX</t>
+        </is>
+      </c>
       <c r="M84" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9316,7 +9468,11 @@
           <t>CTR-720</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
       <c r="J85" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -9327,7 +9483,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>23AAACI1681G1ZX</t>
+        </is>
+      </c>
       <c r="M85" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9415,7 +9575,11 @@
           <t>CTR-721</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>721</t>
+        </is>
+      </c>
       <c r="J86" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -9426,7 +9590,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>08AAACI1681G2ZO</t>
+        </is>
+      </c>
       <c r="M86" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9514,7 +9682,11 @@
           <t>CTR-721</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>721</t>
+        </is>
+      </c>
       <c r="J87" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -9525,7 +9697,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>08AAACI1681G2ZO</t>
+        </is>
+      </c>
       <c r="M87" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9613,7 +9789,11 @@
           <t>CTR-722</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
       <c r="J88" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -9716,7 +9896,11 @@
           <t>CTR-722</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
       <c r="J89" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -9819,7 +10003,11 @@
           <t>CTR-988</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>988</t>
+        </is>
+      </c>
       <c r="J90" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -9830,7 +10018,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M90" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9918,7 +10110,11 @@
           <t>CTR-988</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>988</t>
+        </is>
+      </c>
       <c r="J91" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -9929,7 +10125,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M91" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10017,7 +10217,11 @@
           <t>CTR-989</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>989</t>
+        </is>
+      </c>
       <c r="J92" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -10028,7 +10232,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M92" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10116,7 +10324,11 @@
           <t>CTR-989</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>989</t>
+        </is>
+      </c>
       <c r="J93" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -10127,7 +10339,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>24AAACI1681G1ZV</t>
+        </is>
+      </c>
       <c r="M93" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10215,7 +10431,11 @@
           <t>CTR-990</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>990</t>
+        </is>
+      </c>
       <c r="J94" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -10226,7 +10446,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M94" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10314,7 +10538,11 @@
           <t>CTR-990</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>990</t>
+        </is>
+      </c>
       <c r="J95" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -10325,7 +10553,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M95" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10413,7 +10645,11 @@
           <t>CTR-991</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>991</t>
+        </is>
+      </c>
       <c r="J96" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -10424,7 +10660,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>23AAACI1681G1ZX</t>
+        </is>
+      </c>
       <c r="M96" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10512,7 +10752,11 @@
           <t>CTR-991</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>991</t>
+        </is>
+      </c>
       <c r="J97" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -10523,7 +10767,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>23AAACI1681G1ZX</t>
+        </is>
+      </c>
       <c r="M97" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10611,7 +10859,11 @@
           <t>CTR-992</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>992</t>
+        </is>
+      </c>
       <c r="J98" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -10714,7 +10966,11 @@
           <t>CTR-992</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>992</t>
+        </is>
+      </c>
       <c r="J99" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -10817,7 +11073,11 @@
           <t>CTR-993</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>993</t>
+        </is>
+      </c>
       <c r="J100" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -10828,7 +11088,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>08AAACI1681G2ZO</t>
+        </is>
+      </c>
       <c r="M100" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10916,7 +11180,11 @@
           <t>CTR-993</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>993</t>
+        </is>
+      </c>
       <c r="J101" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -10927,7 +11195,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>08AAACI1681G2ZO</t>
+        </is>
+      </c>
       <c r="M101" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11015,7 +11287,11 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>690</t>
+        </is>
+      </c>
       <c r="J102" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -11026,7 +11302,11 @@
           <t>37AAACR5055K2Z5</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr"/>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M102" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11114,7 +11394,11 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>635</t>
+        </is>
+      </c>
       <c r="J103" t="inlineStr">
         <is>
           <t>AAACR5055K / AAACI1681G</t>
@@ -11217,7 +11501,11 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>635</t>
+        </is>
+      </c>
       <c r="J104" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -11320,7 +11608,11 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>690</t>
+        </is>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>AADCB1672K / AAACI1681G</t>
@@ -11331,7 +11623,11 @@
           <t>37AADCB1672K1ZK</t>
         </is>
       </c>
-      <c r="L105" t="inlineStr"/>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>09AAACI1681G1ZN</t>
+        </is>
+      </c>
       <c r="M105" t="inlineStr">
         <is>
           <t>9.720</t>

</xml_diff>

<commit_message>
Updated UI dashboard and database
</commit_message>
<xml_diff>
--- a/output/invoices.xlsx
+++ b/output/invoices.xlsx
@@ -425,9 +425,9 @@
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
@@ -587,26 +587,10 @@
           <t>3015006421</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>18202884</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -694,26 +678,10 @@
           <t>3016007959</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>18216023</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -801,26 +769,10 @@
           <t>3016007960</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>18216220</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -908,26 +860,10 @@
           <t>3041001254</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>18216025</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1015,26 +951,10 @@
           <t>3041001255</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>18216173</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1122,26 +1042,10 @@
           <t>3041001256</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>18216353</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1229,26 +1133,10 @@
           <t>3040001702</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>18216022</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1336,26 +1224,10 @@
           <t>3040001703</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>18216072</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1443,26 +1315,10 @@
           <t>3040001704</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>18216104</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1550,26 +1406,10 @@
           <t>3040001705</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>18216127</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1657,26 +1497,10 @@
           <t>3040001706</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>18216176</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1764,26 +1588,10 @@
           <t>3040001707</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>18216219</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1871,26 +1679,10 @@
           <t>3040001708</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>18216311</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -1978,26 +1770,10 @@
           <t>3040001709</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>18216355</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -2085,26 +1861,10 @@
           <t>3040001710</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>18216389</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -2192,26 +1952,10 @@
           <t>3040001711</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>18216450</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -2299,26 +2043,10 @@
           <t>3040001712</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>18216535</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -2406,26 +2134,10 @@
           <t>3120015462</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>18215975</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -2513,26 +2225,10 @@
           <t>3120015464</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>18216188</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -2620,26 +2316,10 @@
           <t>3120015467</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>18216336</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -2727,26 +2407,10 @@
           <t>3120015496</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>18215976</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -2834,26 +2498,10 @@
           <t>3120015497</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>18215979</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -2941,26 +2589,10 @@
           <t>3120015498</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>18215981</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -3048,26 +2680,10 @@
           <t>3120015499</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>18216201</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -3155,26 +2771,10 @@
           <t>3120015500</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>18216202</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -3262,26 +2862,10 @@
           <t>3120015501</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>18216208</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>18.42</t>
@@ -3369,26 +2953,10 @@
           <t>3016007961</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>18216030</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -3476,26 +3044,10 @@
           <t>3016007962</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>18216222</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -3583,26 +3135,10 @@
           <t>3016007982</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>18216031</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -3690,26 +3226,10 @@
           <t>3016007983</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>18216223</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -3797,26 +3317,10 @@
           <t>3016007966</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>18216027</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -3904,26 +3408,10 @@
           <t>3016007967</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>18216028</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4011,26 +3499,10 @@
           <t>3016007968</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>18216029</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4118,26 +3590,10 @@
           <t>3016007969</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>18216224</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4225,26 +3681,10 @@
           <t>3016007970</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>18216225</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4332,26 +3772,10 @@
           <t>3016007972</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>18216226</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4439,26 +3863,10 @@
           <t>3060003509</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>18216006</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4546,26 +3954,10 @@
           <t>3060003510</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>18216007</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4653,26 +4045,10 @@
           <t>3060003511</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>18216164</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4760,26 +4136,10 @@
           <t>3060003512</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>18216165</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4867,26 +4227,10 @@
           <t>3060003513</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>18216343</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -4974,26 +4318,10 @@
           <t>3060003516</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>18216346</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5081,26 +4409,10 @@
           <t>3060003514</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>18216008</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5188,26 +4500,10 @@
           <t>3060003515</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>18216167</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5295,26 +4591,10 @@
           <t>3060003517</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>18216347</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5402,26 +4682,10 @@
           <t>3015006423</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>18216035</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5509,26 +4773,10 @@
           <t>3015006424</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>18216036</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5616,26 +4864,10 @@
           <t>3015006425</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>18216229</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5723,26 +4955,10 @@
           <t>3015006426</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>18216230</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
         <is>
           <t>25.63</t>
@@ -5830,26 +5046,10 @@
           <t>3016007979</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>18216024</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -5937,26 +5137,10 @@
           <t>3016007953</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>18202872</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -6044,26 +5228,10 @@
           <t>3016007957</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>18203872</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -6151,26 +5319,10 @@
           <t>3016007958</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>18202871</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -6258,26 +5410,10 @@
           <t>3018018278</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>18202836</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
           <t>96.09</t>
@@ -6365,26 +5501,10 @@
           <t>3043000530</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>18216004</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -6472,26 +5592,10 @@
           <t>3043000531</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>18216284</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>106.77</t>
@@ -6579,26 +5683,10 @@
           <t>3060003507</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>18202904</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -6686,26 +5774,10 @@
           <t>3060003508</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>18204704</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
           <t>80.08</t>
@@ -6793,26 +5865,10 @@
           <t>3110013677</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>18202878</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
           <t>42.04</t>
@@ -6900,26 +5956,10 @@
           <t>3110013678</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>18202879</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>AAACG1209J / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>09AAACG1209J1ZU</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>42.04</t>
@@ -7007,26 +6047,10 @@
           <t>CTR-1246</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>1246</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>10AAACI1681G1Z4</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7114,26 +6138,10 @@
           <t>CTR-1246</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>1246</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>10AAACI1681G1Z4</t>
-        </is>
-      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7221,26 +6229,10 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>635</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>06AAACI1681G1ZT</t>
-        </is>
-      </c>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7328,26 +6320,10 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>635</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>06AAACI1681G1ZT</t>
-        </is>
-      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7435,26 +6411,10 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>690</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7542,26 +6502,10 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>690</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7649,26 +6593,10 @@
           <t>CTR-691</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>691</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7756,26 +6684,10 @@
           <t>CTR-691</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>691</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7863,26 +6775,10 @@
           <t>CTR-692</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>692</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -7970,26 +6866,10 @@
           <t>CTR-692</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>692</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8077,26 +6957,10 @@
           <t>CTR-693</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>693</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8184,26 +7048,10 @@
           <t>CTR-693</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>693</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8291,26 +7139,10 @@
           <t>CTR-694</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>694</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8398,26 +7230,10 @@
           <t>CTR-694</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>694</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8505,26 +7321,10 @@
           <t>CTR-716</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>716</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8612,26 +7412,10 @@
           <t>CTR-716</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>716</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8719,26 +7503,10 @@
           <t>CTR-717</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>717</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8826,26 +7594,10 @@
           <t>CTR-717</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>717</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -8933,26 +7685,10 @@
           <t>CTR-718</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>718</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9040,26 +7776,10 @@
           <t>CTR-718</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>718</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9147,26 +7867,10 @@
           <t>CTR-719</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>719</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9254,26 +7958,10 @@
           <t>CTR-719</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>719</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9361,26 +8049,10 @@
           <t>CTR-720</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>720</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9468,26 +8140,10 @@
           <t>CTR-720</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>720</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9575,26 +8231,10 @@
           <t>CTR-721</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>721</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9682,26 +8322,10 @@
           <t>CTR-721</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>721</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9789,26 +8413,10 @@
           <t>CTR-722</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>722</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -9896,26 +8504,10 @@
           <t>CTR-722</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>722</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10003,26 +8595,10 @@
           <t>CTR-988</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>988</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L90" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10110,26 +8686,10 @@
           <t>CTR-988</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>988</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10217,26 +8777,10 @@
           <t>CTR-989</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>989</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L92" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10324,26 +8868,10 @@
           <t>CTR-989</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>989</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>24AAACI1681G1ZV</t>
-        </is>
-      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10431,26 +8959,10 @@
           <t>CTR-990</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>990</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10538,26 +9050,10 @@
           <t>CTR-990</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>990</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10645,26 +9141,10 @@
           <t>CTR-991</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>991</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10752,26 +9232,10 @@
           <t>CTR-991</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>991</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L97" t="inlineStr">
-        <is>
-          <t>23AAACI1681G1ZX</t>
-        </is>
-      </c>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10859,26 +9323,10 @@
           <t>CTR-992</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>992</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -10966,26 +9414,10 @@
           <t>CTR-992</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>992</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>27AAACI1681G1ZP</t>
-        </is>
-      </c>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11073,26 +9505,10 @@
           <t>CTR-993</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>993</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11180,26 +9596,10 @@
           <t>CTR-993</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>993</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>08AAACI1681G2ZO</t>
-        </is>
-      </c>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11287,26 +9687,10 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>690</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11394,26 +9778,10 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>635</t>
-        </is>
-      </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t>AAACR5055K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K103" t="inlineStr">
-        <is>
-          <t>37AAACR5055K2Z5</t>
-        </is>
-      </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>06AAACI1681G1ZT</t>
-        </is>
-      </c>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11501,26 +9869,10 @@
           <t>CTR-635</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>635</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>06AAACI1681G1ZT</t>
-        </is>
-      </c>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
           <t>9.720</t>
@@ -11608,26 +9960,10 @@
           <t>CTR-690</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>690</t>
-        </is>
-      </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>AADCB1672K / AAACI1681G</t>
-        </is>
-      </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>37AADCB1672K1ZK</t>
-        </is>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>09AAACI1681G1ZN</t>
-        </is>
-      </c>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
           <t>9.720</t>

</xml_diff>